<commit_message>
Smooth wall aero updated and multishot data
</commit_message>
<xml_diff>
--- a/008_COLLINS_FENSAPICE/gridConvergence_D01_V1.xlsx
+++ b/008_COLLINS_FENSAPICE/gridConvergence_D01_V1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\02.IPW3\008_IPW3-main\008_COLLINS_FENSAPICE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1723027-4DA2-424D-ABE9-B6E34A702B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C4688D-57EB-436C-8460-D21C4D45A38A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="661" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="661" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="1" r:id="rId1"/>
@@ -802,6 +802,15 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -821,15 +830,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -856,6 +856,12 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -864,12 +870,6 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2718,36 +2718,36 @@
       <c r="AMG1" s="31"/>
     </row>
     <row r="2" spans="1:1021" s="6" customFormat="1" ht="59.1" customHeight="1">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="68"/>
     </row>
     <row r="3" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
-      <c r="L3" s="52"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="55"/>
       <c r="M3" s="31"/>
       <c r="N3" s="31"/>
       <c r="O3" s="31"/>
@@ -3759,26 +3759,26 @@
       <c r="AMG3" s="31"/>
     </row>
     <row r="4" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="51"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46" t="s">
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
       <c r="M4" s="31"/>
       <c r="N4" s="31"/>
       <c r="O4" s="21"/>
@@ -5053,20 +5053,20 @@
       <c r="N21" s="15"/>
     </row>
     <row r="22" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A22" s="46" t="s">
+      <c r="A22" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
-      <c r="K22" s="46"/>
-      <c r="L22" s="46"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="49"/>
+      <c r="L22" s="49"/>
       <c r="M22" s="33"/>
       <c r="N22" s="33"/>
       <c r="O22" s="31"/>
@@ -6078,26 +6078,26 @@
       <c r="AMG22" s="31"/>
     </row>
     <row r="23" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A23" s="47" t="s">
+      <c r="A23" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="48"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="46" t="s">
+      <c r="B23" s="51"/>
+      <c r="C23" s="52"/>
+      <c r="D23" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46" t="s">
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46" t="s">
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="46"/>
-      <c r="L23" s="46"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
       <c r="M23" s="31"/>
       <c r="N23" s="31"/>
       <c r="O23" s="31"/>
@@ -7370,20 +7370,20 @@
       <c r="L40" s="24"/>
     </row>
     <row r="41" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="67"/>
-      <c r="J41" s="67"/>
-      <c r="K41" s="67"/>
-      <c r="L41" s="67"/>
+      <c r="B41" s="65"/>
+      <c r="C41" s="65"/>
+      <c r="D41" s="65"/>
+      <c r="E41" s="65"/>
+      <c r="F41" s="65"/>
+      <c r="G41" s="65"/>
+      <c r="H41" s="65"/>
+      <c r="I41" s="65"/>
+      <c r="J41" s="65"/>
+      <c r="K41" s="65"/>
+      <c r="L41" s="65"/>
       <c r="M41" s="31"/>
       <c r="N41" s="31"/>
       <c r="O41" s="31"/>
@@ -8395,26 +8395,26 @@
       <c r="AMG41" s="31"/>
     </row>
     <row r="42" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A42" s="47" t="s">
+      <c r="A42" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="48"/>
-      <c r="C42" s="49"/>
-      <c r="D42" s="46" t="s">
+      <c r="B42" s="51"/>
+      <c r="C42" s="52"/>
+      <c r="D42" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46" t="s">
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46" t="s">
+      <c r="H42" s="49"/>
+      <c r="I42" s="49"/>
+      <c r="J42" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
+      <c r="K42" s="49"/>
+      <c r="L42" s="49"/>
       <c r="M42" s="31"/>
       <c r="N42" s="31"/>
       <c r="O42" s="31"/>
@@ -9689,20 +9689,20 @@
       <c r="L59" s="24"/>
     </row>
     <row r="60" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A60" s="67" t="s">
+      <c r="A60" s="65" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="67"/>
-      <c r="C60" s="67"/>
-      <c r="D60" s="67"/>
-      <c r="E60" s="67"/>
-      <c r="F60" s="67"/>
-      <c r="G60" s="67"/>
-      <c r="H60" s="67"/>
-      <c r="I60" s="67"/>
-      <c r="J60" s="67"/>
-      <c r="K60" s="67"/>
-      <c r="L60" s="67"/>
+      <c r="B60" s="65"/>
+      <c r="C60" s="65"/>
+      <c r="D60" s="65"/>
+      <c r="E60" s="65"/>
+      <c r="F60" s="65"/>
+      <c r="G60" s="65"/>
+      <c r="H60" s="65"/>
+      <c r="I60" s="65"/>
+      <c r="J60" s="65"/>
+      <c r="K60" s="65"/>
+      <c r="L60" s="65"/>
       <c r="M60" s="31"/>
       <c r="N60" s="31"/>
       <c r="O60" s="31"/>
@@ -10714,26 +10714,26 @@
       <c r="AMG60" s="31"/>
     </row>
     <row r="61" spans="1:1021" s="32" customFormat="1" ht="26.25">
-      <c r="A61" s="47" t="s">
+      <c r="A61" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="48"/>
-      <c r="C61" s="49"/>
-      <c r="D61" s="46" t="s">
+      <c r="B61" s="51"/>
+      <c r="C61" s="52"/>
+      <c r="D61" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46" t="s">
+      <c r="E61" s="49"/>
+      <c r="F61" s="49"/>
+      <c r="G61" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46" t="s">
+      <c r="H61" s="49"/>
+      <c r="I61" s="49"/>
+      <c r="J61" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="46"/>
-      <c r="L61" s="46"/>
+      <c r="K61" s="49"/>
+      <c r="L61" s="49"/>
       <c r="M61" s="31"/>
       <c r="N61" s="31"/>
       <c r="O61" s="31"/>
@@ -12005,6 +12005,16 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="J61:L61"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="G42:I42"/>
     <mergeCell ref="D1:L1"/>
     <mergeCell ref="J42:L42"/>
     <mergeCell ref="D23:F23"/>
@@ -12017,16 +12027,6 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="A60:L60"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="J61:L61"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="G42:I42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -12050,63 +12050,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="26.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
     </row>
     <row r="2" spans="1:12" s="6" customFormat="1" ht="59.1" customHeight="1">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="68"/>
       <c r="J2" s="45"/>
       <c r="K2" s="45"/>
       <c r="L2" s="45"/>
     </row>
     <row r="3" spans="1:12" ht="26.25">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="52"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="55"/>
     </row>
     <row r="4" spans="1:12" ht="26.25">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="47" t="s">
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="I4" s="49"/>
+      <c r="H4" s="51"/>
+      <c r="I4" s="52"/>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="19" t="s">
@@ -12310,34 +12310,34 @@
       <c r="I13" s="19"/>
     </row>
     <row r="14" spans="1:12" ht="26.25">
-      <c r="A14" s="50" t="s">
+      <c r="A14" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="51"/>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="51"/>
-      <c r="G14" s="51"/>
-      <c r="H14" s="51"/>
-      <c r="I14" s="52"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" spans="1:12" ht="26.25">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46" t="s">
+      <c r="B15" s="49"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="46"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="47" t="s">
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="48"/>
-      <c r="I15" s="49"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="52"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="19" t="s">
@@ -12541,34 +12541,34 @@
       <c r="I24" s="19"/>
     </row>
     <row r="25" spans="1:9" ht="26.25">
-      <c r="A25" s="50" t="s">
+      <c r="A25" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="52"/>
+      <c r="B25" s="54"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
+      <c r="I25" s="55"/>
     </row>
     <row r="26" spans="1:9" ht="26.25">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="46"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46" t="s">
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="46"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="47" t="s">
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="H26" s="48"/>
-      <c r="I26" s="49"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="52"/>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="19" t="s">
@@ -12772,34 +12772,34 @@
       <c r="I35" s="19"/>
     </row>
     <row r="36" spans="1:9" ht="26.25">
-      <c r="A36" s="50" t="s">
+      <c r="A36" s="53" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="51"/>
-      <c r="C36" s="51"/>
-      <c r="D36" s="51"/>
-      <c r="E36" s="51"/>
-      <c r="F36" s="51"/>
-      <c r="G36" s="51"/>
-      <c r="H36" s="51"/>
-      <c r="I36" s="52"/>
+      <c r="B36" s="54"/>
+      <c r="C36" s="54"/>
+      <c r="D36" s="54"/>
+      <c r="E36" s="54"/>
+      <c r="F36" s="54"/>
+      <c r="G36" s="54"/>
+      <c r="H36" s="54"/>
+      <c r="I36" s="55"/>
     </row>
     <row r="37" spans="1:9" ht="26.25">
-      <c r="A37" s="46" t="s">
+      <c r="A37" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="B37" s="46"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="46" t="s">
+      <c r="B37" s="49"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="E37" s="46"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="47" t="s">
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
+      <c r="G37" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="H37" s="48"/>
-      <c r="I37" s="49"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="52"/>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="19" t="s">
@@ -13004,12 +13004,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A36:I36"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="D37:F37"/>
@@ -13022,6 +13016,12 @@
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="D26:F26"/>
     <mergeCell ref="G26:I26"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13066,16 +13066,16 @@
     </row>
     <row r="3" spans="1:1024">
       <c r="A3" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B3" s="11">
-        <v>0.4260331</v>
+        <v>0.47619885000000001</v>
       </c>
       <c r="C3" s="11">
-        <v>2.1593709999999999E-2</v>
+        <v>1.0314814E-2</v>
       </c>
       <c r="D3" s="11">
-        <v>7.1472970000000004E-3</v>
+        <v>1.3165601000000001E-3</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -14140,16 +14140,16 @@
     </row>
     <row r="6" spans="1:1024">
       <c r="A6" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B6" s="11">
-        <v>0.42789949999999999</v>
+        <v>0.47694449999999999</v>
       </c>
       <c r="C6" s="11">
-        <v>2.149506E-2</v>
+        <v>1.0344289E-2</v>
       </c>
       <c r="D6" s="11">
-        <v>6.8521459999999999E-3</v>
+        <v>1.1052135E-3</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -15214,16 +15214,16 @@
     </row>
     <row r="9" spans="1:1024">
       <c r="A9" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B9" s="40">
-        <v>0.42765009999999998</v>
+        <v>0.47528195000000001</v>
       </c>
       <c r="C9" s="40">
-        <v>2.1552970000000001E-2</v>
+        <v>1.0528829E-2</v>
       </c>
       <c r="D9" s="40">
-        <v>6.6363129999999996E-3</v>
+        <v>1.1318540000000001E-3</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -16285,16 +16285,16 @@
     </row>
     <row r="12" spans="1:1024">
       <c r="A12" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B12" s="11">
-        <v>0.43036400000000002</v>
+        <v>0.47658477999999999</v>
       </c>
       <c r="C12" s="11">
-        <v>2.1005570000000001E-2</v>
+        <v>1.1143488999999999E-2</v>
       </c>
       <c r="D12" s="11">
-        <v>6.4524710000000004E-3</v>
+        <v>5.6197577999999996E-4</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -19330,61 +19330,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="26.25">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="55"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="48"/>
     </row>
     <row r="2" spans="1:13" ht="26.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
     </row>
     <row r="3" spans="1:13" ht="26.25">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46" t="s">
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47" t="s">
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="47" t="s">
+      <c r="I3" s="51"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="49"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="52"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="17"/>
@@ -19443,44 +19443,44 @@
       <c r="M5" s="25"/>
     </row>
     <row r="6" spans="1:13" ht="26.25">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="52"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="54"/>
+      <c r="L6" s="54"/>
+      <c r="M6" s="55"/>
     </row>
     <row r="7" spans="1:13" ht="26.25">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46" t="s">
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47" t="s">
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="47" t="s">
+      <c r="I7" s="51"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="48"/>
-      <c r="M7" s="49"/>
+      <c r="L7" s="51"/>
+      <c r="M7" s="52"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="17"/>
@@ -19539,44 +19539,44 @@
       <c r="M9" s="25"/>
     </row>
     <row r="10" spans="1:13" ht="26.25">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
     </row>
     <row r="11" spans="1:13" ht="26.25">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46" t="s">
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47" t="s">
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="48"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="47" t="s">
+      <c r="I11" s="51"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="49"/>
+      <c r="L11" s="51"/>
+      <c r="M11" s="52"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="17"/>
@@ -19635,44 +19635,44 @@
       <c r="M13" s="41"/>
     </row>
     <row r="14" spans="1:13" ht="26.25">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="46"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="46"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:13" ht="26.25">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46" t="s">
+      <c r="B15" s="49"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47" t="s">
+      <c r="F15" s="49"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="48"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="47" t="s">
+      <c r="I15" s="51"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="L15" s="51"/>
+      <c r="M15" s="52"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="17"/>
@@ -19732,6 +19732,16 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="K11:M11"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="A2:M2"/>
@@ -19743,16 +19753,6 @@
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="K7:M7"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="K15:M15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19780,74 +19780,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="26.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
     </row>
     <row r="2" spans="1:17" ht="59.1" customHeight="1">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="68"/>
     </row>
     <row r="3" spans="1:17" s="27" customFormat="1" ht="26.25">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
     </row>
     <row r="4" spans="1:17" s="27" customFormat="1" ht="26.25">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46" t="s">
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
       <c r="N4" s="18"/>
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
@@ -20227,46 +20227,46 @@
       <c r="Q21" s="7"/>
     </row>
     <row r="22" spans="1:17" s="27" customFormat="1" ht="26.25">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="67"/>
-      <c r="C22" s="67"/>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
-      <c r="I22" s="67"/>
-      <c r="J22" s="67"/>
-      <c r="K22" s="67"/>
-      <c r="L22" s="67"/>
+      <c r="B22" s="65"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="65"/>
+      <c r="G22" s="65"/>
+      <c r="H22" s="65"/>
+      <c r="I22" s="65"/>
+      <c r="J22" s="65"/>
+      <c r="K22" s="65"/>
+      <c r="L22" s="65"/>
       <c r="M22" s="28"/>
       <c r="O22" s="29"/>
       <c r="P22" s="29"/>
       <c r="Q22" s="29"/>
     </row>
     <row r="23" spans="1:17" s="27" customFormat="1" ht="26.25">
-      <c r="A23" s="46" t="s">
+      <c r="A23" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46" t="s">
+      <c r="B23" s="49"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46" t="s">
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46" t="s">
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="46"/>
-      <c r="L23" s="46"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
       <c r="O23" s="29"/>
       <c r="P23" s="29"/>
       <c r="Q23" s="29"/>
@@ -20632,45 +20632,45 @@
       <c r="Q40" s="7"/>
     </row>
     <row r="41" spans="1:17" s="27" customFormat="1" ht="26.25">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="67"/>
-      <c r="J41" s="67"/>
-      <c r="K41" s="67"/>
-      <c r="L41" s="67"/>
+      <c r="B41" s="65"/>
+      <c r="C41" s="65"/>
+      <c r="D41" s="65"/>
+      <c r="E41" s="65"/>
+      <c r="F41" s="65"/>
+      <c r="G41" s="65"/>
+      <c r="H41" s="65"/>
+      <c r="I41" s="65"/>
+      <c r="J41" s="65"/>
+      <c r="K41" s="65"/>
+      <c r="L41" s="65"/>
       <c r="O41" s="29"/>
       <c r="P41" s="29"/>
       <c r="Q41" s="29"/>
     </row>
     <row r="42" spans="1:17" s="27" customFormat="1" ht="26.25">
-      <c r="A42" s="46" t="s">
+      <c r="A42" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="46"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46" t="s">
+      <c r="B42" s="49"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46" t="s">
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46" t="s">
+      <c r="H42" s="49"/>
+      <c r="I42" s="49"/>
+      <c r="J42" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
+      <c r="K42" s="49"/>
+      <c r="L42" s="49"/>
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="19" t="s">
@@ -20982,42 +20982,42 @@
       <c r="L59" s="26"/>
     </row>
     <row r="60" spans="1:12" s="27" customFormat="1" ht="26.25">
-      <c r="A60" s="46" t="s">
+      <c r="A60" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="46"/>
-      <c r="C60" s="46"/>
-      <c r="D60" s="46"/>
-      <c r="E60" s="46"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="46"/>
-      <c r="H60" s="46"/>
-      <c r="I60" s="46"/>
-      <c r="J60" s="46"/>
-      <c r="K60" s="46"/>
-      <c r="L60" s="46"/>
+      <c r="B60" s="49"/>
+      <c r="C60" s="49"/>
+      <c r="D60" s="49"/>
+      <c r="E60" s="49"/>
+      <c r="F60" s="49"/>
+      <c r="G60" s="49"/>
+      <c r="H60" s="49"/>
+      <c r="I60" s="49"/>
+      <c r="J60" s="49"/>
+      <c r="K60" s="49"/>
+      <c r="L60" s="49"/>
     </row>
     <row r="61" spans="1:12" s="27" customFormat="1" ht="26.25">
-      <c r="A61" s="46" t="s">
+      <c r="A61" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="46"/>
-      <c r="C61" s="46"/>
-      <c r="D61" s="46" t="s">
+      <c r="B61" s="49"/>
+      <c r="C61" s="49"/>
+      <c r="D61" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46" t="s">
+      <c r="E61" s="49"/>
+      <c r="F61" s="49"/>
+      <c r="G61" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46" t="s">
+      <c r="H61" s="49"/>
+      <c r="I61" s="49"/>
+      <c r="J61" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="46"/>
-      <c r="L61" s="46"/>
+      <c r="K61" s="49"/>
+      <c r="L61" s="49"/>
     </row>
     <row r="62" spans="1:12">
       <c r="A62" s="19" t="s">
@@ -21330,6 +21330,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A42:C42"/>
@@ -21346,12 +21352,6 @@
     <mergeCell ref="D42:F42"/>
     <mergeCell ref="G42:I42"/>
     <mergeCell ref="J42:L42"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="A60:L60"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -21380,61 +21380,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="26.25">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="55"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="48"/>
     </row>
     <row r="2" spans="1:13" ht="26.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
     </row>
     <row r="3" spans="1:13" ht="26.25">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46" t="s">
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47" t="s">
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="47" t="s">
+      <c r="I3" s="51"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="49"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="52"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="17"/>
@@ -21517,44 +21517,44 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="26.25">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="52"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="54"/>
+      <c r="L6" s="54"/>
+      <c r="M6" s="55"/>
     </row>
     <row r="7" spans="1:13" ht="26.25">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46" t="s">
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47" t="s">
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="47" t="s">
+      <c r="I7" s="51"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="48"/>
-      <c r="M7" s="49"/>
+      <c r="L7" s="51"/>
+      <c r="M7" s="52"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="17"/>
@@ -21637,44 +21637,44 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="26.25">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
     </row>
     <row r="11" spans="1:13" ht="26.25">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46" t="s">
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47" t="s">
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="48"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="47" t="s">
+      <c r="I11" s="51"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="49"/>
+      <c r="L11" s="51"/>
+      <c r="M11" s="52"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="17"/>
@@ -21757,44 +21757,44 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="26.25">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="46"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="46"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:13" ht="26.25">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46" t="s">
+      <c r="B15" s="49"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47" t="s">
+      <c r="F15" s="49"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="48"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="47" t="s">
+      <c r="I15" s="51"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="L15" s="51"/>
+      <c r="M15" s="52"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="17"/>
@@ -21878,12 +21878,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -21899,6 +21893,12 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21924,74 +21924,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="26.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
     </row>
     <row r="2" spans="1:12" s="6" customFormat="1" ht="59.1" customHeight="1">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="68"/>
     </row>
     <row r="3" spans="1:12" ht="26.25">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
     </row>
     <row r="4" spans="1:12" ht="26.25">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46" t="s">
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="19" t="s">
@@ -22412,42 +22412,42 @@
       <c r="L21" s="26"/>
     </row>
     <row r="22" spans="1:12" ht="26.25">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="67"/>
-      <c r="C22" s="67"/>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
-      <c r="I22" s="67"/>
-      <c r="J22" s="67"/>
-      <c r="K22" s="67"/>
-      <c r="L22" s="67"/>
+      <c r="B22" s="65"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="65"/>
+      <c r="G22" s="65"/>
+      <c r="H22" s="65"/>
+      <c r="I22" s="65"/>
+      <c r="J22" s="65"/>
+      <c r="K22" s="65"/>
+      <c r="L22" s="65"/>
     </row>
     <row r="23" spans="1:12" ht="26.25">
-      <c r="A23" s="46" t="s">
+      <c r="A23" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46" t="s">
+      <c r="B23" s="49"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46" t="s">
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46" t="s">
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="46"/>
-      <c r="L23" s="46"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="19" t="s">
@@ -22868,42 +22868,42 @@
       <c r="L40" s="26"/>
     </row>
     <row r="41" spans="1:12" ht="26.25">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="67"/>
-      <c r="J41" s="67"/>
-      <c r="K41" s="67"/>
-      <c r="L41" s="67"/>
+      <c r="B41" s="65"/>
+      <c r="C41" s="65"/>
+      <c r="D41" s="65"/>
+      <c r="E41" s="65"/>
+      <c r="F41" s="65"/>
+      <c r="G41" s="65"/>
+      <c r="H41" s="65"/>
+      <c r="I41" s="65"/>
+      <c r="J41" s="65"/>
+      <c r="K41" s="65"/>
+      <c r="L41" s="65"/>
     </row>
     <row r="42" spans="1:12" ht="26.25">
-      <c r="A42" s="46" t="s">
+      <c r="A42" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="46"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46" t="s">
+      <c r="B42" s="49"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46" t="s">
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46" t="s">
+      <c r="H42" s="49"/>
+      <c r="I42" s="49"/>
+      <c r="J42" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
+      <c r="K42" s="49"/>
+      <c r="L42" s="49"/>
     </row>
     <row r="43" spans="1:12">
       <c r="A43" s="19" t="s">
@@ -23324,42 +23324,42 @@
       <c r="L59" s="26"/>
     </row>
     <row r="60" spans="1:12" ht="26.25">
-      <c r="A60" s="46" t="s">
+      <c r="A60" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="46"/>
-      <c r="C60" s="46"/>
-      <c r="D60" s="46"/>
-      <c r="E60" s="46"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="46"/>
-      <c r="H60" s="46"/>
-      <c r="I60" s="46"/>
-      <c r="J60" s="46"/>
-      <c r="K60" s="46"/>
-      <c r="L60" s="46"/>
+      <c r="B60" s="49"/>
+      <c r="C60" s="49"/>
+      <c r="D60" s="49"/>
+      <c r="E60" s="49"/>
+      <c r="F60" s="49"/>
+      <c r="G60" s="49"/>
+      <c r="H60" s="49"/>
+      <c r="I60" s="49"/>
+      <c r="J60" s="49"/>
+      <c r="K60" s="49"/>
+      <c r="L60" s="49"/>
     </row>
     <row r="61" spans="1:12" ht="26.25">
-      <c r="A61" s="46" t="s">
+      <c r="A61" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="46"/>
-      <c r="C61" s="46"/>
-      <c r="D61" s="46" t="s">
+      <c r="B61" s="49"/>
+      <c r="C61" s="49"/>
+      <c r="D61" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46" t="s">
+      <c r="E61" s="49"/>
+      <c r="F61" s="49"/>
+      <c r="G61" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46" t="s">
+      <c r="H61" s="49"/>
+      <c r="I61" s="49"/>
+      <c r="J61" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="46"/>
-      <c r="L61" s="46"/>
+      <c r="K61" s="49"/>
+      <c r="L61" s="49"/>
     </row>
     <row r="62" spans="1:12">
       <c r="A62" s="19" t="s">
@@ -23781,13 +23781,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="A61:C61"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="G61:I61"/>
@@ -23803,6 +23796,13 @@
     <mergeCell ref="G42:I42"/>
     <mergeCell ref="J42:L42"/>
     <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="A2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23829,61 +23829,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="26.25">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
       <c r="M1" s="69"/>
     </row>
     <row r="2" spans="1:13" ht="26.25">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="49"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
+      <c r="L2" s="51"/>
+      <c r="M2" s="52"/>
     </row>
     <row r="3" spans="1:13" s="6" customFormat="1" ht="26.25">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46" t="s">
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47" t="s">
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="47" t="s">
+      <c r="I3" s="51"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="49"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="52"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="38"/>
@@ -23942,44 +23942,44 @@
       <c r="M5" s="39"/>
     </row>
     <row r="6" spans="1:13" ht="26.25">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="49"/>
+      <c r="B6" s="51"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="51"/>
+      <c r="K6" s="51"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="52"/>
     </row>
     <row r="7" spans="1:13" s="6" customFormat="1" ht="26.25">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46" t="s">
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47" t="s">
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="47" t="s">
+      <c r="I7" s="51"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="48"/>
-      <c r="M7" s="49"/>
+      <c r="L7" s="51"/>
+      <c r="M7" s="52"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="38"/>
@@ -24038,44 +24038,44 @@
       <c r="M9" s="25"/>
     </row>
     <row r="10" spans="1:13" ht="26.25">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="48"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="48"/>
-      <c r="K10" s="48"/>
-      <c r="L10" s="48"/>
-      <c r="M10" s="49"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="51"/>
+      <c r="L10" s="51"/>
+      <c r="M10" s="52"/>
     </row>
     <row r="11" spans="1:13" s="6" customFormat="1" ht="26.25">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46" t="s">
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47" t="s">
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="48"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="47" t="s">
+      <c r="I11" s="51"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="49"/>
+      <c r="L11" s="51"/>
+      <c r="M11" s="52"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="38"/>
@@ -24134,44 +24134,44 @@
       <c r="M13" s="41"/>
     </row>
     <row r="14" spans="1:13" ht="26.25">
-      <c r="A14" s="47" t="s">
+      <c r="A14" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="48"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="48"/>
-      <c r="H14" s="48"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="48"/>
-      <c r="K14" s="48"/>
-      <c r="L14" s="48"/>
-      <c r="M14" s="49"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="51"/>
+      <c r="D14" s="51"/>
+      <c r="E14" s="51"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="51"/>
+      <c r="H14" s="51"/>
+      <c r="I14" s="51"/>
+      <c r="J14" s="51"/>
+      <c r="K14" s="51"/>
+      <c r="L14" s="51"/>
+      <c r="M14" s="52"/>
     </row>
     <row r="15" spans="1:13" s="6" customFormat="1" ht="26.25">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46" t="s">
+      <c r="B15" s="49"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47" t="s">
+      <c r="F15" s="49"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="48"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="47" t="s">
+      <c r="I15" s="51"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="L15" s="51"/>
+      <c r="M15" s="52"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="38"/>
@@ -24231,12 +24231,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -24252,6 +24246,12 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>